<commit_message>
Included scripts for geographic mappings for congressional districts for ACS data, wrapped up EIA API requests
</commit_message>
<xml_diff>
--- a/Indicator_Gen/config/CA State Income Brackets by Household Size.xlsx
+++ b/Indicator_Gen/config/CA State Income Brackets by Household Size.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ADDA2A3-C385-4402-B0F1-8DF150E3B085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6E75E3-5C98-44B6-A128-3E74BED18F26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Source" sheetId="3" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="70">
   <si>
     <r>
       <rPr>
@@ -1220,6 +1220,9 @@
   <si>
     <t>Income Limits 2023 (ca.gov)</t>
   </si>
+  <si>
+    <t>HCD</t>
+  </si>
 </sst>
 </file>
 
@@ -1754,7 +1757,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FA59105-81DF-41BE-9D08-0DAA51453A31}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -1763,6 +1766,11 @@
       </c>
       <c r="B1" s="17" t="s">
         <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -12373,48 +12381,6 @@
     </row>
   </sheetData>
   <mergeCells count="58">
-    <mergeCell ref="A14:A19"/>
-    <mergeCell ref="A8:A13"/>
-    <mergeCell ref="A44:A49"/>
-    <mergeCell ref="A38:A43"/>
-    <mergeCell ref="A32:A37"/>
-    <mergeCell ref="A26:A31"/>
-    <mergeCell ref="A20:A25"/>
-    <mergeCell ref="A74:A79"/>
-    <mergeCell ref="A68:A73"/>
-    <mergeCell ref="A62:A67"/>
-    <mergeCell ref="A56:A61"/>
-    <mergeCell ref="A50:A55"/>
-    <mergeCell ref="A104:A109"/>
-    <mergeCell ref="A98:A103"/>
-    <mergeCell ref="A92:A97"/>
-    <mergeCell ref="A86:A91"/>
-    <mergeCell ref="A80:A85"/>
-    <mergeCell ref="A134:A139"/>
-    <mergeCell ref="A128:A133"/>
-    <mergeCell ref="A122:A127"/>
-    <mergeCell ref="A116:A121"/>
-    <mergeCell ref="A110:A115"/>
-    <mergeCell ref="A164:A169"/>
-    <mergeCell ref="A158:A163"/>
-    <mergeCell ref="A152:A157"/>
-    <mergeCell ref="A146:A151"/>
-    <mergeCell ref="A140:A145"/>
-    <mergeCell ref="A194:A199"/>
-    <mergeCell ref="A188:A193"/>
-    <mergeCell ref="A182:A187"/>
-    <mergeCell ref="A176:A181"/>
-    <mergeCell ref="A170:A175"/>
-    <mergeCell ref="A224:A229"/>
-    <mergeCell ref="A218:A223"/>
-    <mergeCell ref="A212:A217"/>
-    <mergeCell ref="A206:A211"/>
-    <mergeCell ref="A200:A205"/>
-    <mergeCell ref="A254:A259"/>
-    <mergeCell ref="A248:A253"/>
-    <mergeCell ref="A242:A247"/>
-    <mergeCell ref="A236:A241"/>
-    <mergeCell ref="A230:A235"/>
     <mergeCell ref="A2:A7"/>
     <mergeCell ref="A344:A349"/>
     <mergeCell ref="A338:A343"/>
@@ -12431,6 +12397,48 @@
     <mergeCell ref="A272:A277"/>
     <mergeCell ref="A266:A271"/>
     <mergeCell ref="A260:A265"/>
+    <mergeCell ref="A254:A259"/>
+    <mergeCell ref="A248:A253"/>
+    <mergeCell ref="A242:A247"/>
+    <mergeCell ref="A236:A241"/>
+    <mergeCell ref="A230:A235"/>
+    <mergeCell ref="A224:A229"/>
+    <mergeCell ref="A218:A223"/>
+    <mergeCell ref="A212:A217"/>
+    <mergeCell ref="A206:A211"/>
+    <mergeCell ref="A200:A205"/>
+    <mergeCell ref="A194:A199"/>
+    <mergeCell ref="A188:A193"/>
+    <mergeCell ref="A182:A187"/>
+    <mergeCell ref="A176:A181"/>
+    <mergeCell ref="A170:A175"/>
+    <mergeCell ref="A164:A169"/>
+    <mergeCell ref="A158:A163"/>
+    <mergeCell ref="A152:A157"/>
+    <mergeCell ref="A146:A151"/>
+    <mergeCell ref="A140:A145"/>
+    <mergeCell ref="A134:A139"/>
+    <mergeCell ref="A128:A133"/>
+    <mergeCell ref="A122:A127"/>
+    <mergeCell ref="A116:A121"/>
+    <mergeCell ref="A110:A115"/>
+    <mergeCell ref="A104:A109"/>
+    <mergeCell ref="A98:A103"/>
+    <mergeCell ref="A92:A97"/>
+    <mergeCell ref="A86:A91"/>
+    <mergeCell ref="A80:A85"/>
+    <mergeCell ref="A74:A79"/>
+    <mergeCell ref="A68:A73"/>
+    <mergeCell ref="A62:A67"/>
+    <mergeCell ref="A56:A61"/>
+    <mergeCell ref="A50:A55"/>
+    <mergeCell ref="A14:A19"/>
+    <mergeCell ref="A8:A13"/>
+    <mergeCell ref="A44:A49"/>
+    <mergeCell ref="A38:A43"/>
+    <mergeCell ref="A32:A37"/>
+    <mergeCell ref="A26:A31"/>
+    <mergeCell ref="A20:A25"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>